<commit_message>
Atualiza respostas processadas, resultados iGovTI, insumos de auditoria e scripts de suporte
</commit_message>
<xml_diff>
--- a/02-Execucao/02-Questionario iGovTI 2023/20260621-comparacao-iGovTI-2023-2026.xlsx
+++ b/02-Execucao/02-Questionario iGovTI 2023/20260621-comparacao-iGovTI-2023-2026.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE70"/>
+  <dimension ref="A1:BE69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12165,12 +12165,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IASERJ</t>
+          <t>UERJ</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>IASERJ</t>
+          <t>UERJ</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -12180,157 +12180,157 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Iniciando</t>
+          <t>Inexpressivo</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Intermediário</t>
+          <t>Inexpressivo</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>0.3940867113248652</v>
+        <v>0.09581582345969374</v>
       </c>
       <c r="H62" t="n">
-        <v>0.4318422865451919</v>
+        <v>0.1023211796921592</v>
       </c>
       <c r="I62" t="n">
-        <v>0.03775557522032674</v>
+        <v>0.006505356232465467</v>
       </c>
       <c r="J62" t="n">
-        <v>0.369136788511888</v>
+        <v>0.09834658780250941</v>
       </c>
       <c r="K62" t="n">
-        <v>0.369136788511888</v>
+        <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>5.551115123125783e-17</v>
+        <v>-0.09834658780250941</v>
       </c>
       <c r="M62" t="n">
-        <v>0.4190366341378423</v>
+        <v>0.09328505911687807</v>
       </c>
       <c r="N62" t="n">
-        <v>0.4945477845784957</v>
+        <v>0.2046423593843184</v>
       </c>
       <c r="O62" t="n">
-        <v>0.07551115044065337</v>
+        <v>0.1113573002674403</v>
       </c>
       <c r="P62" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R62" t="n">
-        <v>0</v>
+        <v>-0.15</v>
       </c>
       <c r="S62" t="n">
-        <v>0.1199770569238325</v>
+        <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>0.1199770569238325</v>
+        <v>0</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
       </c>
       <c r="V62" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="W62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="X62" t="n">
-        <v>0</v>
+        <v>-0.15</v>
       </c>
       <c r="Y62" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="Z62" t="n">
-        <v>0.5</v>
+        <v>0.3125</v>
       </c>
       <c r="AA62" t="n">
-        <v>0</v>
+        <v>0.1625</v>
       </c>
       <c r="AB62" t="n">
-        <v>0.2656285332908624</v>
+        <v>0.07621972903111485</v>
       </c>
       <c r="AC62" t="n">
-        <v>0.5000000000000004</v>
+        <v>0.151309699487875</v>
       </c>
       <c r="AD62" t="n">
-        <v>0.234371466709138</v>
+        <v>0.07508997045676016</v>
       </c>
       <c r="AE62" t="n">
-        <v>0.5000000000000004</v>
+        <v>0.1500000000000001</v>
       </c>
       <c r="AF62" t="n">
-        <v>0.5000000000000004</v>
+        <v>0</v>
       </c>
       <c r="AG62" t="n">
-        <v>0</v>
+        <v>-0.1500000000000001</v>
       </c>
       <c r="AH62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AI62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AJ62" t="n">
         <v>0</v>
       </c>
       <c r="AK62" t="n">
-        <v>0.499999999995</v>
+        <v>0</v>
       </c>
       <c r="AL62" t="n">
-        <v>0.499999999995</v>
+        <v>0</v>
       </c>
       <c r="AM62" t="n">
         <v>0</v>
       </c>
       <c r="AN62" t="n">
-        <v>0.5</v>
+        <v>0.100712374234342</v>
       </c>
       <c r="AO62" t="n">
-        <v>0.5</v>
+        <v>0.2090209092421984</v>
       </c>
       <c r="AP62" t="n">
-        <v>0</v>
+        <v>0.1083085350078564</v>
       </c>
       <c r="AQ62" t="n">
-        <v>0.5</v>
+        <v>0.0230157925124409</v>
       </c>
       <c r="AR62" t="n">
-        <v>0.5</v>
+        <v>0.05275291091015383</v>
       </c>
       <c r="AS62" t="n">
-        <v>0</v>
+        <v>0.02973711839771293</v>
       </c>
       <c r="AT62" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="AU62" t="n">
-        <v>0.5</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="AV62" t="n">
-        <v>0</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="AW62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AX62" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AY62" t="n">
         <v>0</v>
       </c>
       <c r="AZ62" t="n">
-        <v>0.4999999999999995</v>
+        <v>0.1499999999999999</v>
       </c>
       <c r="BA62" t="n">
-        <v>0.4999999999999995</v>
+        <v>0.03677816621792566</v>
       </c>
       <c r="BB62" t="n">
-        <v>0</v>
+        <v>-0.1132218337820742</v>
       </c>
       <c r="BC62" t="inlineStr">
         <is>
@@ -12339,10 +12339,14 @@
       </c>
       <c r="BD62" t="inlineStr">
         <is>
-          <t>Gestão de pessoas de TIC (+0.2344)</t>
-        </is>
-      </c>
-      <c r="BE62" t="inlineStr"/>
+          <t>Processo de software (+0.5667); Planejamento de TIC (+0.1625); Estrutura de segurança da informação (+0.1083)</t>
+        </is>
+      </c>
+      <c r="BE62" t="inlineStr">
+        <is>
+          <t>Gestão de serviços de TIC (-0.1500); Modelo de gestão de TIC (-0.1500); Resultados de TIC (-0.1500)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -12352,12 +12356,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>UERJ</t>
+          <t>EMATER</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>UERJ</t>
+          <t>EMATER</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -12367,171 +12371,171 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
+          <t>Iniciando</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
           <t>Inexpressivo</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Inexpressivo</t>
-        </is>
-      </c>
       <c r="G63" t="n">
-        <v>0.09581582345969374</v>
+        <v>0.2174333044598369</v>
       </c>
       <c r="H63" t="n">
-        <v>0.1023211796921592</v>
+        <v>0.01311539791851239</v>
       </c>
       <c r="I63" t="n">
-        <v>0.006505356232465467</v>
+        <v>-0.2043179065413245</v>
       </c>
       <c r="J63" t="n">
-        <v>0.09834658780250941</v>
+        <v>0.2581768508630193</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>-0.09834658780250941</v>
+        <v>-0.2581768508630193</v>
       </c>
       <c r="M63" t="n">
-        <v>0.09328505911687807</v>
+        <v>0.1766897580566544</v>
       </c>
       <c r="N63" t="n">
-        <v>0.2046423593843184</v>
+        <v>0.02623079583702478</v>
       </c>
       <c r="O63" t="n">
-        <v>0.1113573002674403</v>
+        <v>-0.1504589622196296</v>
       </c>
       <c r="P63" t="n">
-        <v>0.15</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="Q63" t="n">
         <v>0</v>
       </c>
       <c r="R63" t="n">
+        <v>-0.2666666666666667</v>
+      </c>
+      <c r="S63" t="n">
+        <v>0.1889638646550362</v>
+      </c>
+      <c r="T63" t="n">
+        <v>0</v>
+      </c>
+      <c r="U63" t="n">
+        <v>-0.1889638646550362</v>
+      </c>
+      <c r="V63" t="n">
+        <v>0.3250000000000001</v>
+      </c>
+      <c r="W63" t="n">
+        <v>0</v>
+      </c>
+      <c r="X63" t="n">
+        <v>-0.3250000000000001</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>-0.125</v>
+      </c>
+      <c r="AB63" t="n">
+        <v>0.1500000000000001</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>0.0569729761117809</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>-0.09302702388821923</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>0.2420350108418368</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG63" t="n">
+        <v>-0.2420350108418368</v>
+      </c>
+      <c r="AH63" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AI63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ63" t="n">
         <v>-0.15</v>
       </c>
-      <c r="S63" t="n">
-        <v>0</v>
-      </c>
-      <c r="T63" t="n">
-        <v>0</v>
-      </c>
-      <c r="U63" t="n">
-        <v>0</v>
-      </c>
-      <c r="V63" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="W63" t="n">
-        <v>0</v>
-      </c>
-      <c r="X63" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="Y63" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Z63" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="AA63" t="n">
-        <v>0.1625</v>
-      </c>
-      <c r="AB63" t="n">
-        <v>0.07621972903111485</v>
-      </c>
-      <c r="AC63" t="n">
-        <v>0.151309699487875</v>
-      </c>
-      <c r="AD63" t="n">
-        <v>0.07508997045676016</v>
-      </c>
-      <c r="AE63" t="n">
-        <v>0.1500000000000001</v>
-      </c>
-      <c r="AF63" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG63" t="n">
-        <v>-0.1500000000000001</v>
-      </c>
-      <c r="AH63" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI63" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ63" t="n">
-        <v>0</v>
-      </c>
       <c r="AK63" t="n">
-        <v>0</v>
+        <v>0.17602635035325</v>
       </c>
       <c r="AL63" t="n">
         <v>0</v>
       </c>
       <c r="AM63" t="n">
-        <v>0</v>
+        <v>-0.17602635035325</v>
       </c>
       <c r="AN63" t="n">
-        <v>0.100712374234342</v>
+        <v>0.3819712053403692</v>
       </c>
       <c r="AO63" t="n">
-        <v>0.2090209092421984</v>
+        <v>0</v>
       </c>
       <c r="AP63" t="n">
-        <v>0.1083085350078564</v>
+        <v>-0.3819712053403692</v>
       </c>
       <c r="AQ63" t="n">
-        <v>0.0230157925124409</v>
+        <v>0.1803573783995376</v>
       </c>
       <c r="AR63" t="n">
-        <v>0.05275291091015383</v>
+        <v>0.04504181142414375</v>
       </c>
       <c r="AS63" t="n">
-        <v>0.02973711839771293</v>
+        <v>-0.1353155669753939</v>
       </c>
       <c r="AT63" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="AU63" t="n">
-        <v>0.7166666666666667</v>
+        <v>0</v>
       </c>
       <c r="AV63" t="n">
-        <v>0.5666666666666667</v>
+        <v>-0.05</v>
       </c>
       <c r="AW63" t="n">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="AX63" t="n">
         <v>0</v>
       </c>
       <c r="AY63" t="n">
-        <v>0</v>
+        <v>-0.49</v>
       </c>
       <c r="AZ63" t="n">
+        <v>0.1332826517191245</v>
+      </c>
+      <c r="BA63" t="n">
         <v>0.1499999999999999</v>
       </c>
-      <c r="BA63" t="n">
-        <v>0.03677816621792566</v>
-      </c>
       <c r="BB63" t="n">
-        <v>-0.1132218337820742</v>
+        <v>0.01671734828087537</v>
       </c>
       <c r="BC63" t="inlineStr">
         <is>
-          <t>avanço</t>
+          <t>regressão</t>
         </is>
       </c>
       <c r="BD63" t="inlineStr">
         <is>
-          <t>Processo de software (+0.5667); Planejamento de TIC (+0.1625); Estrutura de segurança da informação (+0.1083)</t>
+          <t>Processos de contratação de TIC (+0.0167)</t>
         </is>
       </c>
       <c r="BE63" t="inlineStr">
         <is>
-          <t>Gestão de serviços de TIC (-0.1500); Modelo de gestão de TIC (-0.1500); Resultados de TIC (-0.1500)</t>
+          <t>Gestão de projetos de TIC (-0.4900); Estrutura de segurança da informação (-0.3820); Resultados de TIC (-0.3250)</t>
         </is>
       </c>
     </row>
@@ -12543,12 +12547,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EMATER</t>
+          <t>FLXIII</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>EMATER</t>
+          <t>FLXIII</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -12567,148 +12571,148 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>0.2174333044598369</v>
+        <v>0.1751499683786731</v>
       </c>
       <c r="H64" t="n">
-        <v>0.01311539791851239</v>
+        <v>0.09506818522245383</v>
       </c>
       <c r="I64" t="n">
-        <v>-0.2043179065413245</v>
+        <v>-0.08008178315621928</v>
       </c>
       <c r="J64" t="n">
-        <v>0.2581768508630193</v>
+        <v>0.2168535966847315</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>0.160711053811857</v>
       </c>
       <c r="L64" t="n">
-        <v>-0.2581768508630193</v>
+        <v>-0.05614254287287454</v>
       </c>
       <c r="M64" t="n">
-        <v>0.1766897580566544</v>
+        <v>0.1334463400726147</v>
       </c>
       <c r="N64" t="n">
-        <v>0.02623079583702478</v>
+        <v>0.02942531663305064</v>
       </c>
       <c r="O64" t="n">
-        <v>-0.1504589622196296</v>
+        <v>-0.104021023439564</v>
       </c>
       <c r="P64" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="Q64" t="n">
         <v>0</v>
       </c>
       <c r="R64" t="n">
-        <v>-0.2666666666666667</v>
+        <v>-0.5</v>
       </c>
       <c r="S64" t="n">
-        <v>0.1889638646550362</v>
+        <v>0.08698336626977857</v>
       </c>
       <c r="T64" t="n">
-        <v>0</v>
+        <v>0.01199770569238325</v>
       </c>
       <c r="U64" t="n">
-        <v>-0.1889638646550362</v>
+        <v>-0.07498566057739532</v>
       </c>
       <c r="V64" t="n">
-        <v>0.3250000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="W64" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="X64" t="n">
-        <v>-0.3250000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="Y64" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="Z64" t="n">
         <v>0.025</v>
       </c>
       <c r="AA64" t="n">
-        <v>-0.125</v>
+        <v>-0.225</v>
       </c>
       <c r="AB64" t="n">
-        <v>0.1500000000000001</v>
+        <v>0.0389925511800589</v>
       </c>
       <c r="AC64" t="n">
-        <v>0.0569729761117809</v>
+        <v>0.02429690983669855</v>
       </c>
       <c r="AD64" t="n">
-        <v>-0.09302702388821923</v>
+        <v>-0.01469564134336035</v>
       </c>
       <c r="AE64" t="n">
-        <v>0.2420350108418368</v>
+        <v>0.0264027476415732</v>
       </c>
       <c r="AF64" t="n">
-        <v>0</v>
+        <v>0.0381845691462976</v>
       </c>
       <c r="AG64" t="n">
-        <v>-0.2420350108418368</v>
+        <v>0.0117818215047244</v>
       </c>
       <c r="AH64" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="AI64" t="n">
         <v>0</v>
       </c>
       <c r="AJ64" t="n">
-        <v>-0.15</v>
+        <v>-0.5</v>
       </c>
       <c r="AK64" t="n">
-        <v>0.17602635035325</v>
+        <v>0.0687416456475</v>
       </c>
       <c r="AL64" t="n">
-        <v>0</v>
+        <v>0.0499999999995</v>
       </c>
       <c r="AM64" t="n">
-        <v>-0.17602635035325</v>
+        <v>-0.018741645648</v>
       </c>
       <c r="AN64" t="n">
-        <v>0.3819712053403692</v>
+        <v>0.167095350315001</v>
       </c>
       <c r="AO64" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="AP64" t="n">
-        <v>-0.3819712053403692</v>
+        <v>-0.117095350315001</v>
       </c>
       <c r="AQ64" t="n">
-        <v>0.1803573783995376</v>
+        <v>0.04504181142414375</v>
       </c>
       <c r="AR64" t="n">
-        <v>0.04504181142414375</v>
+        <v>0.02481049554247315</v>
       </c>
       <c r="AS64" t="n">
-        <v>-0.1353155669753939</v>
+        <v>-0.0202313158816706</v>
       </c>
       <c r="AT64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU64" t="n">
         <v>0.05</v>
       </c>
-      <c r="AU64" t="n">
-        <v>0</v>
-      </c>
       <c r="AV64" t="n">
-        <v>-0.05</v>
+        <v>0.05</v>
       </c>
       <c r="AW64" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="AX64" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="AY64" t="n">
-        <v>-0.49</v>
+        <v>0.05</v>
       </c>
       <c r="AZ64" t="n">
-        <v>0.1332826517191245</v>
+        <v>0.3142858778741451</v>
       </c>
       <c r="BA64" t="n">
-        <v>0.1499999999999999</v>
+        <v>0</v>
       </c>
       <c r="BB64" t="n">
-        <v>0.01671734828087537</v>
+        <v>-0.3142858778741451</v>
       </c>
       <c r="BC64" t="inlineStr">
         <is>
@@ -12717,12 +12721,12 @@
       </c>
       <c r="BD64" t="inlineStr">
         <is>
-          <t>Processos de contratação de TIC (+0.0167)</t>
+          <t>Resultados de TIC (+0.4500); Processo de software (+0.0500); Gestão de projetos de TIC (+0.0500)</t>
         </is>
       </c>
       <c r="BE64" t="inlineStr">
         <is>
-          <t>Gestão de projetos de TIC (-0.4900); Estrutura de segurança da informação (-0.3820); Resultados de TIC (-0.3250)</t>
+          <t>Gestão de níveis de serviço (-0.5000); Modelo de gestão de TIC (-0.5000); Processos de contratação de TIC (-0.3143)</t>
         </is>
       </c>
     </row>
@@ -12734,12 +12738,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>FLXIII</t>
+          <t>LOTERJ</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FLXIII</t>
+          <t>LOTERJ</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -12758,148 +12762,148 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>0.1751499683786731</v>
+        <v>0.1857445177631775</v>
       </c>
       <c r="H65" t="n">
-        <v>0.09506818522245383</v>
+        <v>0.0546824815763732</v>
       </c>
       <c r="I65" t="n">
-        <v>-0.08008178315621928</v>
+        <v>-0.1310620361868043</v>
       </c>
       <c r="J65" t="n">
-        <v>0.2168535966847315</v>
+        <v>0.177835292656543</v>
       </c>
       <c r="K65" t="n">
-        <v>0.160711053811857</v>
+        <v>0.06263182835793522</v>
       </c>
       <c r="L65" t="n">
-        <v>-0.05614254287287454</v>
+        <v>-0.1152034642986078</v>
       </c>
       <c r="M65" t="n">
-        <v>0.1334463400726147</v>
+        <v>0.193653742869812</v>
       </c>
       <c r="N65" t="n">
-        <v>0.02942531663305064</v>
+        <v>0.04673313479481117</v>
       </c>
       <c r="O65" t="n">
-        <v>-0.104021023439564</v>
+        <v>-0.1469206080750009</v>
       </c>
       <c r="P65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="S65" t="n">
+        <v>0.01199770569238325</v>
+      </c>
+      <c r="T65" t="n">
+        <v>0</v>
+      </c>
+      <c r="U65" t="n">
+        <v>-0.01199770569238325</v>
+      </c>
+      <c r="V65" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R65" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="S65" t="n">
-        <v>0.08698336626977857</v>
-      </c>
-      <c r="T65" t="n">
-        <v>0.01199770569238325</v>
-      </c>
-      <c r="U65" t="n">
-        <v>-0.07498566057739532</v>
-      </c>
-      <c r="V65" t="n">
+      <c r="W65" t="n">
+        <v>0.2000000000000001</v>
+      </c>
+      <c r="X65" t="n">
+        <v>-0.2999999999999999</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Z65" t="n">
         <v>0.05</v>
       </c>
-      <c r="W65" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="X65" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Y65" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Z65" t="n">
-        <v>0.025</v>
-      </c>
       <c r="AA65" t="n">
-        <v>-0.225</v>
+        <v>-0.09999999999999999</v>
       </c>
       <c r="AB65" t="n">
-        <v>0.0389925511800589</v>
+        <v>0.3087020859827003</v>
       </c>
       <c r="AC65" t="n">
-        <v>0.02429690983669855</v>
+        <v>0.0251270729411436</v>
       </c>
       <c r="AD65" t="n">
-        <v>-0.01469564134336035</v>
+        <v>-0.2835750130415567</v>
       </c>
       <c r="AE65" t="n">
-        <v>0.0264027476415732</v>
+        <v>0.1500000000000001</v>
       </c>
       <c r="AF65" t="n">
-        <v>0.0381845691462976</v>
+        <v>0.1000734209092133</v>
       </c>
       <c r="AG65" t="n">
-        <v>0.0117818215047244</v>
+        <v>-0.04992657909078684</v>
       </c>
       <c r="AH65" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="AI65" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="AJ65" t="n">
-        <v>-0.5</v>
+        <v>-0.09999999999999999</v>
       </c>
       <c r="AK65" t="n">
-        <v>0.0687416456475</v>
+        <v>0.1499999999985</v>
       </c>
       <c r="AL65" t="n">
         <v>0.0499999999995</v>
       </c>
       <c r="AM65" t="n">
-        <v>-0.018741645648</v>
+        <v>-0.099999999999</v>
       </c>
       <c r="AN65" t="n">
-        <v>0.167095350315001</v>
+        <v>0.05058376913984175</v>
       </c>
       <c r="AO65" t="n">
-        <v>0.05</v>
+        <v>0.1633070482397685</v>
       </c>
       <c r="AP65" t="n">
-        <v>-0.117095350315001</v>
+        <v>0.1127232790999267</v>
       </c>
       <c r="AQ65" t="n">
-        <v>0.04504181142414375</v>
+        <v>0.176175188687523</v>
       </c>
       <c r="AR65" t="n">
-        <v>0.02481049554247315</v>
+        <v>0.2268692448455959</v>
       </c>
       <c r="AS65" t="n">
-        <v>-0.0202313158816706</v>
+        <v>0.05069405615807293</v>
       </c>
       <c r="AT65" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="AU65" t="n">
         <v>0.05</v>
       </c>
       <c r="AV65" t="n">
-        <v>0.05</v>
+        <v>-0.09999999999999999</v>
       </c>
       <c r="AW65" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="AX65" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="AY65" t="n">
-        <v>0.05</v>
+        <v>-0.15</v>
       </c>
       <c r="AZ65" t="n">
-        <v>0.3142858778741451</v>
+        <v>0.886322031690047</v>
       </c>
       <c r="BA65" t="n">
-        <v>0</v>
+        <v>0.08191500657628896</v>
       </c>
       <c r="BB65" t="n">
-        <v>-0.3142858778741451</v>
+        <v>-0.8044070251137581</v>
       </c>
       <c r="BC65" t="inlineStr">
         <is>
@@ -12908,29 +12912,29 @@
       </c>
       <c r="BD65" t="inlineStr">
         <is>
-          <t>Resultados de TIC (+0.4500); Processo de software (+0.0500); Gestão de projetos de TIC (+0.0500)</t>
+          <t>Estrutura de segurança da informação (+0.1127); Processos de segurança da informação (+0.0507)</t>
         </is>
       </c>
       <c r="BE65" t="inlineStr">
         <is>
-          <t>Gestão de níveis de serviço (-0.5000); Modelo de gestão de TIC (-0.5000); Processos de contratação de TIC (-0.3143)</t>
+          <t>Processos de contratação de TIC (-0.8044); Resultados de TIC (-0.3000); Gestão de pessoas de TIC (-0.2836)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Estaduais</t>
+          <t>Municípios</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LOTERJ</t>
+          <t>PREFEITURA MUNICIPAL DE MARICA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>LOTERJ</t>
+          <t>MARICÁ</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -12945,44 +12949,44 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Inexpressivo</t>
+          <t>Iniciando</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>0.1857445177631775</v>
+        <v>0.1706500856580512</v>
       </c>
       <c r="H66" t="n">
-        <v>0.0546824815763732</v>
+        <v>0.2006770758047239</v>
       </c>
       <c r="I66" t="n">
-        <v>-0.1310620361868043</v>
+        <v>0.03002699014667268</v>
       </c>
       <c r="J66" t="n">
-        <v>0.177835292656543</v>
+        <v>0.1823911853280631</v>
       </c>
       <c r="K66" t="n">
-        <v>0.06263182835793522</v>
+        <v>0.2751326745723582</v>
       </c>
       <c r="L66" t="n">
-        <v>-0.1152034642986078</v>
+        <v>0.09274148924429509</v>
       </c>
       <c r="M66" t="n">
-        <v>0.193653742869812</v>
+        <v>0.1589089859880394</v>
       </c>
       <c r="N66" t="n">
-        <v>0.04673313479481117</v>
+        <v>0.1262214770370897</v>
       </c>
       <c r="O66" t="n">
-        <v>-0.1469206080750009</v>
+        <v>-0.03268750895094968</v>
       </c>
       <c r="P66" t="n">
-        <v>0.05</v>
+        <v>0.3833333333333334</v>
       </c>
       <c r="Q66" t="n">
         <v>0</v>
       </c>
       <c r="R66" t="n">
-        <v>-0.05</v>
+        <v>-0.3833333333333334</v>
       </c>
       <c r="S66" t="n">
         <v>0.01199770569238325</v>
@@ -12994,13 +12998,13 @@
         <v>-0.01199770569238325</v>
       </c>
       <c r="V66" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="W66" t="n">
-        <v>0.2000000000000001</v>
+        <v>0.8785714285714286</v>
       </c>
       <c r="X66" t="n">
-        <v>-0.2999999999999999</v>
+        <v>0.7285714285714285</v>
       </c>
       <c r="Y66" t="n">
         <v>0.15</v>
@@ -13012,99 +13016,99 @@
         <v>-0.09999999999999999</v>
       </c>
       <c r="AB66" t="n">
-        <v>0.3087020859827003</v>
+        <v>0.0189909920372603</v>
       </c>
       <c r="AC66" t="n">
-        <v>0.0251270729411436</v>
+        <v>0</v>
       </c>
       <c r="AD66" t="n">
-        <v>-0.2835750130415567</v>
+        <v>-0.0189909920372603</v>
       </c>
       <c r="AE66" t="n">
-        <v>0.1500000000000001</v>
+        <v>0.6752003695409512</v>
       </c>
       <c r="AF66" t="n">
-        <v>0.1000734209092133</v>
+        <v>0.6426216813895063</v>
       </c>
       <c r="AG66" t="n">
-        <v>-0.04992657909078684</v>
+        <v>-0.03257868815144493</v>
       </c>
       <c r="AH66" t="n">
-        <v>0.15</v>
+        <v>0.3833333333333334</v>
       </c>
       <c r="AI66" t="n">
-        <v>0.05</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="AJ66" t="n">
-        <v>-0.09999999999999999</v>
+        <v>0.04999999999999993</v>
       </c>
       <c r="AK66" t="n">
-        <v>0.1499999999985</v>
+        <v>0.0958277637645</v>
       </c>
       <c r="AL66" t="n">
-        <v>0.0499999999995</v>
+        <v>0.0229138818825</v>
       </c>
       <c r="AM66" t="n">
-        <v>-0.099999999999</v>
+        <v>-0.072913881882</v>
       </c>
       <c r="AN66" t="n">
-        <v>0.05058376913984175</v>
+        <v>0.01686125637994725</v>
       </c>
       <c r="AO66" t="n">
-        <v>0.1633070482397685</v>
+        <v>0.1224079851365004</v>
       </c>
       <c r="AP66" t="n">
-        <v>0.1127232790999267</v>
+        <v>0.1055467287565532</v>
       </c>
       <c r="AQ66" t="n">
-        <v>0.176175188687523</v>
+        <v>0.1135781376919435</v>
       </c>
       <c r="AR66" t="n">
-        <v>0.2268692448455959</v>
+        <v>0.4463913798207021</v>
       </c>
       <c r="AS66" t="n">
-        <v>0.05069405615807293</v>
+        <v>0.3328132421287586</v>
       </c>
       <c r="AT66" t="n">
-        <v>0.15</v>
+        <v>0.2958333333333334</v>
       </c>
       <c r="AU66" t="n">
-        <v>0.05</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="AV66" t="n">
-        <v>-0.09999999999999999</v>
+        <v>-0.02916666666666667</v>
       </c>
       <c r="AW66" t="n">
         <v>0.15</v>
       </c>
       <c r="AX66" t="n">
-        <v>0</v>
+        <v>0.2375</v>
       </c>
       <c r="AY66" t="n">
-        <v>-0.15</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="AZ66" t="n">
-        <v>0.886322031690047</v>
+        <v>0.04922153598202701</v>
       </c>
       <c r="BA66" t="n">
-        <v>0.08191500657628896</v>
+        <v>0.943161015845023</v>
       </c>
       <c r="BB66" t="n">
-        <v>-0.8044070251137581</v>
+        <v>0.8939394798629959</v>
       </c>
       <c r="BC66" t="inlineStr">
         <is>
-          <t>regressão</t>
+          <t>avanço</t>
         </is>
       </c>
       <c r="BD66" t="inlineStr">
         <is>
-          <t>Estrutura de segurança da informação (+0.1127); Processos de segurança da informação (+0.0507)</t>
+          <t>Processos de contratação de TIC (+0.8939); Resultados de TIC (+0.7286); Processos de segurança da informação (+0.3328)</t>
         </is>
       </c>
       <c r="BE66" t="inlineStr">
         <is>
-          <t>Processos de contratação de TIC (-0.8044); Resultados de TIC (-0.3000); Gestão de pessoas de TIC (-0.2836)</t>
+          <t>Modelo de gestão de TIC (-0.3833); Planejamento de TIC (-0.1000); Gestão de riscos de TIC (-0.0729)</t>
         </is>
       </c>
     </row>
@@ -13116,12 +13120,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE MARICA</t>
+          <t>PREFEITURA MUNICIPAL DE RIO DAS OSTRAS</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MARICÁ</t>
+          <t>RIO DAS OSTRAS</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -13131,157 +13135,157 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
+          <t>Inexpressivo</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
           <t>Iniciando</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Iniciando</t>
-        </is>
-      </c>
       <c r="G67" t="n">
-        <v>0.1706500856580512</v>
+        <v>0.05898448949927405</v>
       </c>
       <c r="H67" t="n">
-        <v>0.2006770758047239</v>
+        <v>0.190282824014711</v>
       </c>
       <c r="I67" t="n">
-        <v>0.03002699014667268</v>
+        <v>0.1312983345154369</v>
       </c>
       <c r="J67" t="n">
-        <v>0.1823911853280631</v>
+        <v>0.0156579570894838</v>
       </c>
       <c r="K67" t="n">
-        <v>0.2751326745723582</v>
+        <v>0.3094633429076835</v>
       </c>
       <c r="L67" t="n">
-        <v>0.09274148924429509</v>
+        <v>0.2938053858181997</v>
       </c>
       <c r="M67" t="n">
-        <v>0.1589089859880394</v>
+        <v>0.1023110219090643</v>
       </c>
       <c r="N67" t="n">
-        <v>0.1262214770370897</v>
+        <v>0.07110230512173854</v>
       </c>
       <c r="O67" t="n">
-        <v>-0.03268750895094968</v>
+        <v>-0.03120871678732576</v>
       </c>
       <c r="P67" t="n">
-        <v>0.3833333333333334</v>
+        <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="R67" t="n">
-        <v>-0.3833333333333334</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="S67" t="n">
-        <v>0.01199770569238325</v>
+        <v>0</v>
       </c>
       <c r="T67" t="n">
         <v>0</v>
       </c>
       <c r="U67" t="n">
-        <v>-0.01199770569238325</v>
+        <v>0</v>
       </c>
       <c r="V67" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="W67" t="n">
-        <v>0.8785714285714286</v>
+        <v>0.5142857142857142</v>
       </c>
       <c r="X67" t="n">
-        <v>0.7285714285714285</v>
+        <v>0.4642857142857142</v>
       </c>
       <c r="Y67" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Z67" t="n">
+        <v>0.14375</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>0.14375</v>
+      </c>
+      <c r="AB67" t="n">
+        <v>0.127715490388402</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>0.008990212465861</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>-0.118725277922541</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>0.2594577447794352</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>0.0515800977033492</v>
+      </c>
+      <c r="AG67" t="n">
+        <v>-0.207877647076086</v>
+      </c>
+      <c r="AH67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI67" t="n">
         <v>0.05</v>
       </c>
-      <c r="AA67" t="n">
-        <v>-0.09999999999999999</v>
-      </c>
-      <c r="AB67" t="n">
-        <v>0.0189909920372603</v>
-      </c>
-      <c r="AC67" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD67" t="n">
-        <v>-0.0189909920372603</v>
-      </c>
-      <c r="AE67" t="n">
-        <v>0.6752003695409512</v>
-      </c>
-      <c r="AF67" t="n">
-        <v>0.6426216813895063</v>
-      </c>
-      <c r="AG67" t="n">
-        <v>-0.03257868815144493</v>
-      </c>
-      <c r="AH67" t="n">
-        <v>0.3833333333333334</v>
-      </c>
-      <c r="AI67" t="n">
-        <v>0.4333333333333333</v>
-      </c>
       <c r="AJ67" t="n">
-        <v>0.04999999999999993</v>
+        <v>0.05</v>
       </c>
       <c r="AK67" t="n">
-        <v>0.0958277637645</v>
+        <v>0</v>
       </c>
       <c r="AL67" t="n">
         <v>0.0229138818825</v>
       </c>
       <c r="AM67" t="n">
-        <v>-0.072913881882</v>
+        <v>0.0229138818825</v>
       </c>
       <c r="AN67" t="n">
-        <v>0.01686125637994725</v>
+        <v>0.1214010459356202</v>
       </c>
       <c r="AO67" t="n">
-        <v>0.1224079851365004</v>
+        <v>0.1410507844517152</v>
       </c>
       <c r="AP67" t="n">
-        <v>0.1055467287565532</v>
+        <v>0.019649738516095</v>
       </c>
       <c r="AQ67" t="n">
-        <v>0.1135781376919435</v>
+        <v>0.3136545176288784</v>
       </c>
       <c r="AR67" t="n">
-        <v>0.4463913798207021</v>
+        <v>0.4180982828107959</v>
       </c>
       <c r="AS67" t="n">
-        <v>0.3328132421287586</v>
+        <v>0.1044437651819175</v>
       </c>
       <c r="AT67" t="n">
-        <v>0.2958333333333334</v>
+        <v>0.3250000000000001</v>
       </c>
       <c r="AU67" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.05</v>
       </c>
       <c r="AV67" t="n">
-        <v>-0.02916666666666667</v>
+        <v>-0.2750000000000001</v>
       </c>
       <c r="AW67" t="n">
         <v>0.15</v>
       </c>
       <c r="AX67" t="n">
-        <v>0.2375</v>
+        <v>0</v>
       </c>
       <c r="AY67" t="n">
-        <v>0.08749999999999999</v>
+        <v>-0.15</v>
       </c>
       <c r="AZ67" t="n">
-        <v>0.04922153598202701</v>
+        <v>0.9715805079225109</v>
       </c>
       <c r="BA67" t="n">
-        <v>0.943161015845023</v>
+        <v>0.6547658145877073</v>
       </c>
       <c r="BB67" t="n">
-        <v>0.8939394798629959</v>
+        <v>-0.3168146933348036</v>
       </c>
       <c r="BC67" t="inlineStr">
         <is>
@@ -13290,12 +13294,12 @@
       </c>
       <c r="BD67" t="inlineStr">
         <is>
-          <t>Processos de contratação de TIC (+0.8939); Resultados de TIC (+0.7286); Processos de segurança da informação (+0.3328)</t>
+          <t>Resultados de TIC (+0.4643); Modelo de gestão de TIC (+0.4333); Planejamento de TIC (+0.1437)</t>
         </is>
       </c>
       <c r="BE67" t="inlineStr">
         <is>
-          <t>Modelo de gestão de TIC (-0.3833); Planejamento de TIC (-0.1000); Gestão de riscos de TIC (-0.0729)</t>
+          <t>Processos de contratação de TIC (-0.3168); Processo de software (-0.2750); Gestão de serviços de TIC (-0.2079)</t>
         </is>
       </c>
     </row>
@@ -13307,12 +13311,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE RIO DAS OSTRAS</t>
+          <t>PREFEITURA MUNICIPAL DE SAQUAREMA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>RIO DAS OSTRAS</t>
+          <t>SAQUAREMA</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -13327,166 +13331,166 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Iniciando</t>
+          <t>Inexpressivo</t>
         </is>
       </c>
       <c r="G68" t="n">
-        <v>0.05898448949927405</v>
+        <v>0.08974221849947667</v>
       </c>
       <c r="H68" t="n">
-        <v>0.190282824014711</v>
+        <v>0.017062113299654</v>
       </c>
       <c r="I68" t="n">
-        <v>0.1312983345154369</v>
+        <v>-0.07268010519982267</v>
       </c>
       <c r="J68" t="n">
-        <v>0.0156579570894838</v>
+        <v>0.06376716528511499</v>
       </c>
       <c r="K68" t="n">
-        <v>0.3094633429076835</v>
+        <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>0.2938053858181997</v>
+        <v>-0.06376716528511499</v>
       </c>
       <c r="M68" t="n">
-        <v>0.1023110219090643</v>
+        <v>0.1157172717138383</v>
       </c>
       <c r="N68" t="n">
-        <v>0.07110230512173854</v>
+        <v>0.034124226599308</v>
       </c>
       <c r="O68" t="n">
-        <v>-0.03120871678732576</v>
+        <v>-0.08159304511453035</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.4333333333333333</v>
+        <v>0</v>
       </c>
       <c r="R68" t="n">
-        <v>0.4333333333333333</v>
+        <v>-0.15</v>
       </c>
       <c r="S68" t="n">
-        <v>0</v>
+        <v>0.03599311707714975</v>
       </c>
       <c r="T68" t="n">
         <v>0</v>
       </c>
       <c r="U68" t="n">
-        <v>0</v>
+        <v>-0.03599311707714975</v>
       </c>
       <c r="V68" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="W68" t="n">
-        <v>0.5142857142857142</v>
+        <v>0</v>
       </c>
       <c r="X68" t="n">
-        <v>0.4642857142857142</v>
+        <v>0</v>
       </c>
       <c r="Y68" t="n">
-        <v>0</v>
+        <v>0.075</v>
       </c>
       <c r="Z68" t="n">
-        <v>0.14375</v>
+        <v>0</v>
       </c>
       <c r="AA68" t="n">
-        <v>0.14375</v>
+        <v>-0.075</v>
       </c>
       <c r="AB68" t="n">
-        <v>0.127715490388402</v>
+        <v>0.1311010408671301</v>
       </c>
       <c r="AC68" t="n">
-        <v>0.008990212465861</v>
+        <v>0.0300023387141979</v>
       </c>
       <c r="AD68" t="n">
-        <v>-0.118725277922541</v>
+        <v>-0.1010987021529322</v>
       </c>
       <c r="AE68" t="n">
-        <v>0.2594577447794352</v>
+        <v>0.3114187484378689</v>
       </c>
       <c r="AF68" t="n">
-        <v>0.0515800977033492</v>
+        <v>0.07511013136381997</v>
       </c>
       <c r="AG68" t="n">
-        <v>-0.207877647076086</v>
+        <v>-0.236308617074049</v>
       </c>
       <c r="AH68" t="n">
-        <v>0</v>
+        <v>0.3833333333333334</v>
       </c>
       <c r="AI68" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.05</v>
+        <v>-0.3833333333333334</v>
       </c>
       <c r="AK68" t="n">
-        <v>0</v>
+        <v>0.0687416456475</v>
       </c>
       <c r="AL68" t="n">
-        <v>0.0229138818825</v>
+        <v>0.108840938941875</v>
       </c>
       <c r="AM68" t="n">
-        <v>0.0229138818825</v>
+        <v>0.040099293294375</v>
       </c>
       <c r="AN68" t="n">
-        <v>0.1214010459356202</v>
+        <v>0.05058376913984175</v>
       </c>
       <c r="AO68" t="n">
-        <v>0.1410507844517152</v>
+        <v>0</v>
       </c>
       <c r="AP68" t="n">
-        <v>0.019649738516095</v>
+        <v>-0.05058376913984175</v>
       </c>
       <c r="AQ68" t="n">
-        <v>0.3136545176288784</v>
+        <v>0.102608969461302</v>
       </c>
       <c r="AR68" t="n">
-        <v>0.4180982828107959</v>
+        <v>0.0795931769488611</v>
       </c>
       <c r="AS68" t="n">
-        <v>0.1044437651819175</v>
+        <v>-0.0230157925124409</v>
       </c>
       <c r="AT68" t="n">
-        <v>0.3250000000000001</v>
+        <v>0</v>
       </c>
       <c r="AU68" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="AV68" t="n">
-        <v>-0.2750000000000001</v>
+        <v>0.15</v>
       </c>
       <c r="AW68" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AX68" t="n">
         <v>0</v>
       </c>
       <c r="AY68" t="n">
-        <v>-0.15</v>
+        <v>0</v>
       </c>
       <c r="AZ68" t="n">
-        <v>0.9715805079225109</v>
+        <v>0.1499999999999999</v>
       </c>
       <c r="BA68" t="n">
-        <v>0.6547658145877073</v>
+        <v>0.1249239775786869</v>
       </c>
       <c r="BB68" t="n">
-        <v>-0.3168146933348036</v>
+        <v>-0.02507602242131296</v>
       </c>
       <c r="BC68" t="inlineStr">
         <is>
-          <t>avanço</t>
+          <t>regressão</t>
         </is>
       </c>
       <c r="BD68" t="inlineStr">
         <is>
-          <t>Resultados de TIC (+0.4643); Modelo de gestão de TIC (+0.4333); Planejamento de TIC (+0.1437)</t>
+          <t>Processo de software (+0.1500); Gestão de riscos de TIC (+0.0401)</t>
         </is>
       </c>
       <c r="BE68" t="inlineStr">
         <is>
-          <t>Processos de contratação de TIC (-0.3168); Processo de software (-0.2750); Gestão de serviços de TIC (-0.2079)</t>
+          <t>Gestão de níveis de serviço (-0.3833); Gestão de serviços de TIC (-0.2363); Modelo de gestão de TIC (-0.1500)</t>
         </is>
       </c>
     </row>
@@ -13498,12 +13502,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE SAQUAREMA</t>
+          <t>PREFEITURA MUNICIPAL DE VOLTA REDONDA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SAQUAREMA</t>
+          <t>VOLTA REDONDA</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -13522,103 +13526,103 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>0.08974221849947667</v>
+        <v>0.06174532745203043</v>
       </c>
       <c r="H69" t="n">
-        <v>0.017062113299654</v>
+        <v>0.003131375757495653</v>
       </c>
       <c r="I69" t="n">
-        <v>-0.07268010519982267</v>
+        <v>-0.05861395169453477</v>
       </c>
       <c r="J69" t="n">
-        <v>0.06376716528511499</v>
+        <v>0.0469738712684514</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
       </c>
       <c r="L69" t="n">
-        <v>-0.06376716528511499</v>
+        <v>-0.0469738712684514</v>
       </c>
       <c r="M69" t="n">
-        <v>0.1157172717138383</v>
+        <v>0.07651678363560946</v>
       </c>
       <c r="N69" t="n">
-        <v>0.034124226599308</v>
+        <v>0.006262751514991307</v>
       </c>
       <c r="O69" t="n">
-        <v>-0.08159304511453035</v>
+        <v>-0.07025403212061815</v>
       </c>
       <c r="P69" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Q69" t="n">
         <v>0</v>
       </c>
       <c r="R69" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="W69" t="n">
+        <v>0</v>
+      </c>
+      <c r="X69" t="n">
         <v>-0.15</v>
       </c>
-      <c r="S69" t="n">
-        <v>0.03599311707714975</v>
-      </c>
-      <c r="T69" t="n">
-        <v>0</v>
-      </c>
-      <c r="U69" t="n">
-        <v>-0.03599311707714975</v>
-      </c>
-      <c r="V69" t="n">
-        <v>0</v>
-      </c>
-      <c r="W69" t="n">
-        <v>0</v>
-      </c>
-      <c r="X69" t="n">
-        <v>0</v>
-      </c>
       <c r="Y69" t="n">
-        <v>0.075</v>
+        <v>0</v>
       </c>
       <c r="Z69" t="n">
         <v>0</v>
       </c>
       <c r="AA69" t="n">
-        <v>-0.075</v>
+        <v>0</v>
       </c>
       <c r="AB69" t="n">
-        <v>0.1311010408671301</v>
+        <v>0.1275631085206467</v>
       </c>
       <c r="AC69" t="n">
-        <v>0.0300023387141979</v>
+        <v>0.02079301917136905</v>
       </c>
       <c r="AD69" t="n">
-        <v>-0.1010987021529322</v>
+        <v>-0.1067700893492777</v>
       </c>
       <c r="AE69" t="n">
-        <v>0.3114187484378689</v>
+        <v>0.08453721549745902</v>
       </c>
       <c r="AF69" t="n">
-        <v>0.07511013136381997</v>
+        <v>0</v>
       </c>
       <c r="AG69" t="n">
-        <v>-0.236308617074049</v>
+        <v>-0.08453721549745902</v>
       </c>
       <c r="AH69" t="n">
-        <v>0.3833333333333334</v>
+        <v>0.15</v>
       </c>
       <c r="AI69" t="n">
         <v>0</v>
       </c>
       <c r="AJ69" t="n">
-        <v>-0.3833333333333334</v>
+        <v>-0.15</v>
       </c>
       <c r="AK69" t="n">
-        <v>0.0687416456475</v>
+        <v>0.081258354351</v>
       </c>
       <c r="AL69" t="n">
-        <v>0.108840938941875</v>
+        <v>0</v>
       </c>
       <c r="AM69" t="n">
-        <v>0.040099293294375</v>
+        <v>-0.081258354351</v>
       </c>
       <c r="AN69" t="n">
         <v>0.05058376913984175</v>
@@ -13630,239 +13634,48 @@
         <v>-0.05058376913984175</v>
       </c>
       <c r="AQ69" t="n">
-        <v>0.102608969461302</v>
+        <v>0.05255272086013965</v>
       </c>
       <c r="AR69" t="n">
-        <v>0.0795931769488611</v>
+        <v>0</v>
       </c>
       <c r="AS69" t="n">
-        <v>-0.0230157925124409</v>
+        <v>-0.05255272086013965</v>
       </c>
       <c r="AT69" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="AU69" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AV69" t="n">
-        <v>0.15</v>
+        <v>-0.15</v>
       </c>
       <c r="AW69" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="AX69" t="n">
         <v>0</v>
       </c>
       <c r="AY69" t="n">
-        <v>0</v>
+        <v>-0.15</v>
       </c>
       <c r="AZ69" t="n">
-        <v>0.1499999999999999</v>
+        <v>0.04086286184158935</v>
       </c>
       <c r="BA69" t="n">
-        <v>0.1249239775786869</v>
+        <v>0.02507602242131295</v>
       </c>
       <c r="BB69" t="n">
-        <v>-0.02507602242131296</v>
+        <v>-0.0157868394202764</v>
       </c>
       <c r="BC69" t="inlineStr">
         <is>
           <t>regressão</t>
         </is>
       </c>
-      <c r="BD69" t="inlineStr">
-        <is>
-          <t>Processo de software (+0.1500); Gestão de riscos de TIC (+0.0401)</t>
-        </is>
-      </c>
+      <c r="BD69" t="inlineStr"/>
       <c r="BE69" t="inlineStr">
-        <is>
-          <t>Gestão de níveis de serviço (-0.3833); Gestão de serviços de TIC (-0.2363); Modelo de gestão de TIC (-0.1500)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Municípios</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>PREFEITURA MUNICIPAL DE VOLTA REDONDA</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>VOLTA REDONDA</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>normalizado</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Inexpressivo</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Inexpressivo</t>
-        </is>
-      </c>
-      <c r="G70" t="n">
-        <v>0.06174532745203043</v>
-      </c>
-      <c r="H70" t="n">
-        <v>0.003131375757495653</v>
-      </c>
-      <c r="I70" t="n">
-        <v>-0.05861395169453477</v>
-      </c>
-      <c r="J70" t="n">
-        <v>0.0469738712684514</v>
-      </c>
-      <c r="K70" t="n">
-        <v>0</v>
-      </c>
-      <c r="L70" t="n">
-        <v>-0.0469738712684514</v>
-      </c>
-      <c r="M70" t="n">
-        <v>0.07651678363560946</v>
-      </c>
-      <c r="N70" t="n">
-        <v>0.006262751514991307</v>
-      </c>
-      <c r="O70" t="n">
-        <v>-0.07025403212061815</v>
-      </c>
-      <c r="P70" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q70" t="n">
-        <v>0</v>
-      </c>
-      <c r="R70" t="n">
-        <v>0</v>
-      </c>
-      <c r="S70" t="n">
-        <v>0</v>
-      </c>
-      <c r="T70" t="n">
-        <v>0</v>
-      </c>
-      <c r="U70" t="n">
-        <v>0</v>
-      </c>
-      <c r="V70" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="W70" t="n">
-        <v>0</v>
-      </c>
-      <c r="X70" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="Y70" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB70" t="n">
-        <v>0.1275631085206467</v>
-      </c>
-      <c r="AC70" t="n">
-        <v>0.02079301917136905</v>
-      </c>
-      <c r="AD70" t="n">
-        <v>-0.1067700893492777</v>
-      </c>
-      <c r="AE70" t="n">
-        <v>0.08453721549745902</v>
-      </c>
-      <c r="AF70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG70" t="n">
-        <v>-0.08453721549745902</v>
-      </c>
-      <c r="AH70" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="AI70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ70" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AK70" t="n">
-        <v>0.081258354351</v>
-      </c>
-      <c r="AL70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM70" t="n">
-        <v>-0.081258354351</v>
-      </c>
-      <c r="AN70" t="n">
-        <v>0.05058376913984175</v>
-      </c>
-      <c r="AO70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP70" t="n">
-        <v>-0.05058376913984175</v>
-      </c>
-      <c r="AQ70" t="n">
-        <v>0.05255272086013965</v>
-      </c>
-      <c r="AR70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS70" t="n">
-        <v>-0.05255272086013965</v>
-      </c>
-      <c r="AT70" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="AU70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV70" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AW70" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="AX70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY70" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="AZ70" t="n">
-        <v>0.04086286184158935</v>
-      </c>
-      <c r="BA70" t="n">
-        <v>0.02507602242131295</v>
-      </c>
-      <c r="BB70" t="n">
-        <v>-0.0157868394202764</v>
-      </c>
-      <c r="BC70" t="inlineStr">
-        <is>
-          <t>regressão</t>
-        </is>
-      </c>
-      <c r="BD70" t="inlineStr"/>
-      <c r="BE70" t="inlineStr">
         <is>
           <t>Gestão de níveis de serviço (-0.1500); Gestão de projetos de TIC (-0.1500); Processo de software (-0.1500)</t>
         </is>
@@ -13921,10 +13734,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C2" t="n">
         <v>36</v>
@@ -13933,7 +13746,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
         <v>16</v>
@@ -14025,25 +13838,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1832169657987048</v>
+        <v>0.1801159401292025</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1462705456010846</v>
+        <v>0.1419437973010805</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1880790071180739</v>
+        <v>0.1844942530088516</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1316501605441191</v>
+        <v>0.1302145646224835</v>
       </c>
       <c r="G2" t="n">
-        <v>0.004862041319369068</v>
+        <v>0.004378312879649103</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.003465539215846691</v>
+        <v>-0.003615056546364903</v>
       </c>
       <c r="I2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J2" t="n">
         <v>36</v>
@@ -14064,22 +13877,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1543652979930324</v>
+        <v>0.1512068937206963</v>
       </c>
       <c r="D3" t="n">
         <v>0.1107410365535664</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1631824569866691</v>
+        <v>0.1601537168171806</v>
       </c>
       <c r="F3" t="n">
-        <v>0.09834658780250941</v>
+        <v>0.09799077653095961</v>
       </c>
       <c r="G3" t="n">
-        <v>0.008817158993636628</v>
+        <v>0.008946823096484225</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>-0.004320705738215636</v>
       </c>
       <c r="I3" t="n">
         <v>31</v>
@@ -14088,7 +13901,7 @@
         <v>34</v>
       </c>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -14103,25 +13916,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.2120686336043772</v>
+        <v>0.2090249865377087</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1678782289885298</v>
+        <v>0.1633936074882846</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2129755572494788</v>
+        <v>0.2088347892005226</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1541200166044084</v>
+        <v>0.1533631689949307</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0009069236451015115</v>
+        <v>-0.000190197337186016</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.01442889218445605</v>
+        <v>-0.01486210988396745</v>
       </c>
       <c r="I4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J4" t="n">
         <v>36</v>
@@ -14142,19 +13955,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.1822866344605475</v>
+        <v>0.1776143790849673</v>
       </c>
       <c r="D5" t="n">
         <v>0.15</v>
       </c>
       <c r="E5" t="n">
-        <v>0.207085346215781</v>
+        <v>0.2027777777777778</v>
       </c>
       <c r="F5" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.02479871175523349</v>
+        <v>0.02516339869281045</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -14166,7 +13979,7 @@
         <v>29</v>
       </c>
       <c r="K5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -14181,19 +13994,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.07839554307320559</v>
+        <v>0.07778405022246106</v>
       </c>
       <c r="D6" t="n">
         <v>0.03599311707714975</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1016635442625</v>
+        <v>0.1013942278998334</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02326800118929445</v>
+        <v>0.02361017767737231</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -14205,7 +14018,7 @@
         <v>29</v>
       </c>
       <c r="K6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -14220,22 +14033,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.2073671497584541</v>
+        <v>0.2030637254901961</v>
       </c>
       <c r="D7" t="n">
         <v>0.15</v>
       </c>
       <c r="E7" t="n">
-        <v>0.182815734989648</v>
+        <v>0.1781512605042017</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.02455141476880607</v>
+        <v>-0.02491246498599439</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>-0.025</v>
       </c>
       <c r="I7" t="n">
         <v>19</v>
@@ -14244,7 +14057,7 @@
         <v>34</v>
       </c>
       <c r="K7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -14259,19 +14072,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.2963681849551414</v>
+        <v>0.2933735994397759</v>
       </c>
       <c r="D8" t="n">
         <v>0.15</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3771014492753623</v>
+        <v>0.3752941176470588</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3125</v>
+        <v>0.3</v>
       </c>
       <c r="G8" t="n">
-        <v>0.08073326432022085</v>
+        <v>0.08192051820728292</v>
       </c>
       <c r="H8" t="n">
         <v>0.025</v>
@@ -14283,7 +14096,7 @@
         <v>25</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -14298,25 +14111,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.2032921939429229</v>
+        <v>0.202375483070159</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1311010408671301</v>
+        <v>0.1310651629461775</v>
       </c>
       <c r="E9" t="n">
-        <v>0.06636625024357881</v>
+        <v>0.05998928333539615</v>
       </c>
       <c r="F9" t="n">
         <v>0.0300023387141979</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.136925943699344</v>
+        <v>-0.1423861997347629</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.0954179496589326</v>
+        <v>-0.09825832590593242</v>
       </c>
       <c r="I9" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J9" t="n">
         <v>51</v>
@@ -14337,22 +14150,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.1546607833614552</v>
+        <v>0.1495822654697119</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1160254158557815</v>
+        <v>0.1056736956852704</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1770009452274486</v>
+        <v>0.1722509591278523</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1021091197076115</v>
+        <v>0.1010912703084124</v>
       </c>
       <c r="G10" t="n">
-        <v>0.02234016186599339</v>
+        <v>0.02266869365814035</v>
       </c>
       <c r="H10" t="n">
-        <v>6.938893903907228e-18</v>
+        <v>0.001033627972744717</v>
       </c>
       <c r="I10" t="n">
         <v>34</v>
@@ -14361,7 +14174,7 @@
         <v>31</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -14376,19 +14189,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.1214975845410628</v>
+        <v>0.1159313725490196</v>
       </c>
       <c r="D11" t="n">
-        <v>0.05</v>
+        <v>0.025</v>
       </c>
       <c r="E11" t="n">
-        <v>0.09710144927536231</v>
+        <v>0.0911764705882353</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.02439613526570048</v>
+        <v>-0.02475490196078431</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -14400,7 +14213,7 @@
         <v>23</v>
       </c>
       <c r="K11" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -14415,19 +14228,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.1065587943408522</v>
+        <v>0.100772894257703</v>
       </c>
       <c r="D12" t="n">
-        <v>0.081258354351</v>
+        <v>0.07499999999925</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1718355734563098</v>
+        <v>0.1670096260072114</v>
       </c>
       <c r="F12" t="n">
         <v>0.081258354351</v>
       </c>
       <c r="G12" t="n">
-        <v>0.06527677911545764</v>
+        <v>0.06623673174950846</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -14439,7 +14252,7 @@
         <v>25</v>
       </c>
       <c r="K12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -14454,22 +14267,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.1366552669145238</v>
+        <v>0.131311962016208</v>
       </c>
       <c r="D13" t="n">
         <v>0.05058376913984175</v>
       </c>
       <c r="E13" t="n">
-        <v>0.271018831833527</v>
+        <v>0.2676514617134319</v>
       </c>
       <c r="F13" t="n">
         <v>0.1591957468445924</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1343635649190032</v>
+        <v>0.1363394996972238</v>
       </c>
       <c r="H13" t="n">
-        <v>0.06698986147444755</v>
+        <v>0.06830646205284899</v>
       </c>
       <c r="I13" t="n">
         <v>43</v>
@@ -14478,7 +14291,7 @@
         <v>19</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -14493,22 +14306,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.1765470074822684</v>
+        <v>0.1717903458275959</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1246269636009447</v>
+        <v>0.1212478595974801</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2171719975700906</v>
+        <v>0.213012762240239</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1738630250995395</v>
+        <v>0.1721345106125336</v>
       </c>
       <c r="G14" t="n">
-        <v>0.04062499008782221</v>
+        <v>0.04122241641264313</v>
       </c>
       <c r="H14" t="n">
-        <v>0.02973711839771293</v>
+        <v>0.03138064401758772</v>
       </c>
       <c r="I14" t="n">
         <v>38</v>
@@ -14517,7 +14330,7 @@
         <v>28</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -14532,19 +14345,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.1998792270531401</v>
+        <v>0.1954656862745098</v>
       </c>
       <c r="D15" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2381642512077295</v>
+        <v>0.2343137254901961</v>
       </c>
       <c r="F15" t="n">
         <v>0.15</v>
       </c>
       <c r="G15" t="n">
-        <v>0.03828502415458937</v>
+        <v>0.03884803921568628</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -14556,7 +14369,7 @@
         <v>22</v>
       </c>
       <c r="K15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -14571,19 +14384,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.1473913043478261</v>
+        <v>0.1422058823529412</v>
       </c>
       <c r="D16" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2195652173913044</v>
+        <v>0.2154411764705882</v>
       </c>
       <c r="F16" t="n">
         <v>0.15</v>
       </c>
       <c r="G16" t="n">
-        <v>0.07217391304347824</v>
+        <v>0.07323529411764704</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -14595,7 +14408,7 @@
         <v>17</v>
       </c>
       <c r="K16" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -14610,22 +14423,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.457236917495524</v>
+        <v>0.4566080486351641</v>
       </c>
       <c r="D17" t="n">
-        <v>0.382580965277926</v>
+        <v>0.3820685911901328</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2504801944701473</v>
+        <v>0.2468107855652965</v>
       </c>
       <c r="F17" t="n">
         <v>0.1249239775786869</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.2067567230253768</v>
+        <v>-0.2097972630698677</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.2241922064938677</v>
+        <v>-0.2278742117981037</v>
       </c>
       <c r="I17" t="n">
         <v>17</v>
@@ -14634,7 +14447,7 @@
         <v>48</v>
       </c>
       <c r="K17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -14710,7 +14523,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -27027,178 +26840,66 @@
           <t>IASERJ</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>IASERJ</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>IASERJ</t>
-        </is>
-      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>normalizado</t>
+          <t>sem correspondência</t>
         </is>
       </c>
       <c r="G70" t="b">
-        <v>1</v>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>Iniciando</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Intermediário</t>
-        </is>
-      </c>
-      <c r="J70" t="n">
-        <v>0.3940867113248652</v>
-      </c>
-      <c r="K70" t="n">
-        <v>0.4318422865451919</v>
-      </c>
-      <c r="L70" t="n">
-        <v>0.03775557522032674</v>
-      </c>
-      <c r="M70" t="n">
-        <v>0.369136788511888</v>
-      </c>
-      <c r="N70" t="n">
-        <v>0.369136788511888</v>
-      </c>
-      <c r="O70" t="n">
-        <v>5.551115123125783e-17</v>
-      </c>
-      <c r="P70" t="n">
-        <v>0.4190366341378423</v>
-      </c>
-      <c r="Q70" t="n">
-        <v>0.4945477845784957</v>
-      </c>
-      <c r="R70" t="n">
-        <v>0.07551115044065337</v>
-      </c>
-      <c r="S70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="U70" t="n">
-        <v>0</v>
-      </c>
-      <c r="V70" t="n">
-        <v>0.1199770569238325</v>
-      </c>
-      <c r="W70" t="n">
-        <v>0.1199770569238325</v>
-      </c>
-      <c r="X70" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Z70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AA70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AC70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AD70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE70" t="n">
-        <v>0.2656285332908624</v>
-      </c>
-      <c r="AF70" t="n">
-        <v>0.5000000000000004</v>
-      </c>
-      <c r="AG70" t="n">
-        <v>0.234371466709138</v>
-      </c>
-      <c r="AH70" t="n">
-        <v>0.5000000000000004</v>
-      </c>
-      <c r="AI70" t="n">
-        <v>0.5000000000000004</v>
-      </c>
-      <c r="AJ70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AL70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AM70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN70" t="n">
-        <v>0.499999999995</v>
-      </c>
-      <c r="AO70" t="n">
-        <v>0.499999999995</v>
-      </c>
-      <c r="AP70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AR70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AS70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AU70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AV70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AX70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AY70" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="BA70" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="BB70" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC70" t="n">
-        <v>0.4999999999999995</v>
-      </c>
-      <c r="BD70" t="n">
-        <v>0.4999999999999995</v>
-      </c>
-      <c r="BE70" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr"/>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr"/>
+      <c r="AD70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AF70" t="inlineStr"/>
+      <c r="AG70" t="inlineStr"/>
+      <c r="AH70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr"/>
+      <c r="AJ70" t="inlineStr"/>
+      <c r="AK70" t="inlineStr"/>
+      <c r="AL70" t="inlineStr"/>
+      <c r="AM70" t="inlineStr"/>
+      <c r="AN70" t="inlineStr"/>
+      <c r="AO70" t="inlineStr"/>
+      <c r="AP70" t="inlineStr"/>
+      <c r="AQ70" t="inlineStr"/>
+      <c r="AR70" t="inlineStr"/>
+      <c r="AS70" t="inlineStr"/>
+      <c r="AT70" t="inlineStr"/>
+      <c r="AU70" t="inlineStr"/>
+      <c r="AV70" t="inlineStr"/>
+      <c r="AW70" t="inlineStr"/>
+      <c r="AX70" t="inlineStr"/>
+      <c r="AY70" t="inlineStr"/>
+      <c r="AZ70" t="inlineStr"/>
+      <c r="BA70" t="inlineStr"/>
+      <c r="BB70" t="inlineStr"/>
+      <c r="BC70" t="inlineStr"/>
+      <c r="BD70" t="inlineStr"/>
+      <c r="BE70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -28800,7 +28501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE10"/>
+  <dimension ref="A1:BE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29714,12 +29415,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SEPOL</t>
+          <t>IASERJ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SEPOL</t>
+          <t>IASERJ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -29783,6 +29484,83 @@
       <c r="BD10" t="inlineStr"/>
       <c r="BE10" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Estaduais</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SEPOL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SEPOL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sem correspondência</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>